<commit_message>
Cap nhat Tam hoa 2026-08-22
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lịch sử" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lịch sử" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hướng dẫn" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -555,30 +555,30 @@
     </row>
     <row r="5">
       <c r="A5" s="29" t="n">
-        <v>46256.57744307289</v>
+        <v>46256.58521197497</v>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>13:51:31</t>
+          <t>14:02:42</t>
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D5" s="30" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E5" s="30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" s="30" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G5" s="30" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H5" s="31" t="n">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-08-23
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -12,8 +12,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -143,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -198,6 +199,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -472,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -555,7 +563,7 @@
     </row>
     <row r="5">
       <c r="A5" s="29" t="n">
-        <v>46256.95055730196</v>
+        <v>46256.95055730324</v>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
@@ -586,6 +594,44 @@
         </is>
       </c>
       <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="32" t="n">
+        <v>46257.95165781066</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>22:50:23</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="n">
+        <v>314</v>
+      </c>
+      <c r="D6" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="33" t="n">
+        <v>248</v>
+      </c>
+      <c r="F6" s="34" t="n">
+        <v>527</v>
+      </c>
+      <c r="G6" s="33" t="n">
+        <v>36</v>
+      </c>
+      <c r="H6" s="33" t="n">
+        <v>150</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-08-24
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -601,7 +601,7 @@
     </row>
     <row r="6">
       <c r="A6" s="32" t="n">
-        <v>46257.95165781066</v>
+        <v>46257.9516578125</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -632,6 +632,44 @@
         </is>
       </c>
       <c r="J6" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="32" t="n">
+        <v>46259.00320925877</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>00:04:37</t>
+        </is>
+      </c>
+      <c r="C7" s="34" t="n">
+        <v>473</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>92</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>407</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>54</v>
+      </c>
+      <c r="G7" s="33" t="n">
+        <v>82</v>
+      </c>
+      <c r="H7" s="33" t="n">
+        <v>23</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-08-25
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,7 @@
     </row>
     <row r="7">
       <c r="A7" s="32" t="n">
-        <v>46259.00320925877</v>
+        <v>46259.00320925926</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -670,6 +670,44 @@
         </is>
       </c>
       <c r="J7" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="n">
+        <v>46260.00359671941</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>00:05:10</t>
+        </is>
+      </c>
+      <c r="C8" s="34" t="n">
+        <v>632</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <v>39</v>
+      </c>
+      <c r="E8" s="33" t="n">
+        <v>156</v>
+      </c>
+      <c r="F8" s="33" t="n">
+        <v>83</v>
+      </c>
+      <c r="G8" s="33" t="n">
+        <v>96</v>
+      </c>
+      <c r="H8" s="33" t="n">
+        <v>182</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-08-28
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -677,7 +677,7 @@
     </row>
     <row r="8">
       <c r="A8" s="32" t="n">
-        <v>46260.00359671941</v>
+        <v>46260.00359672453</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -708,6 +708,44 @@
         </is>
       </c>
       <c r="J8" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="n">
+        <v>46262.33428326609</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:01:22</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="n">
+        <v>970</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>377</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>95</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <v>421</v>
+      </c>
+      <c r="G9" s="33" t="n">
+        <v>213</v>
+      </c>
+      <c r="H9" s="33" t="n">
+        <v>231</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-08-29
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -12,9 +12,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -753,30 +752,30 @@
     </row>
     <row r="10">
       <c r="A10" s="32" t="n">
-        <v>46263.2072598732</v>
+        <v>46263.9216319522</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:58:27</t>
-        </is>
-      </c>
-      <c r="C10" s="34" t="n">
-        <v>1109</v>
+          <t>22:07:09</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="n">
+        <v>59</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" s="33" t="n">
-        <v>234</v>
+        <v>29</v>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>393</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>560</v>
+        <v>96</v>
       </c>
       <c r="G10" s="33" t="n">
-        <v>73</v>
+        <v>232</v>
       </c>
       <c r="H10" s="33" t="n">
-        <v>59</v>
+        <v>218</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-08-30
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -12,8 +12,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -479,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -752,7 +753,7 @@
     </row>
     <row r="10">
       <c r="A10" s="32" t="n">
-        <v>46263.9216319522</v>
+        <v>46263.92163195602</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -783,6 +784,44 @@
         </is>
       </c>
       <c r="J10" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="32" t="n">
+        <v>46264.92174448814</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>22:07:18</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>40</v>
+      </c>
+      <c r="D11" s="33" t="n">
+        <v>110</v>
+      </c>
+      <c r="E11" s="34" t="n">
+        <v>552</v>
+      </c>
+      <c r="F11" s="33" t="n">
+        <v>255</v>
+      </c>
+      <c r="G11" s="33" t="n">
+        <v>84</v>
+      </c>
+      <c r="H11" s="33" t="n">
+        <v>156</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-08-31
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -791,7 +791,7 @@
     </row>
     <row r="11">
       <c r="A11" s="32" t="n">
-        <v>46264.92174448814</v>
+        <v>46264.92174449074</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -822,6 +822,44 @@
         </is>
       </c>
       <c r="J11" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="32" t="n">
+        <v>46265.92161601769</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>22:07:07</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="n">
+        <v>199</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <v>269</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>711</v>
+      </c>
+      <c r="F12" s="33" t="n">
+        <v>414</v>
+      </c>
+      <c r="G12" s="33" t="n">
+        <v>67</v>
+      </c>
+      <c r="H12" s="33" t="n">
+        <v>315</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-01
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -829,7 +829,7 @@
     </row>
     <row r="12">
       <c r="A12" s="32" t="n">
-        <v>46265.92161601769</v>
+        <v>46265.92161601852</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -860,6 +860,44 @@
         </is>
       </c>
       <c r="J12" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="32" t="n">
+        <v>46266.92584414461</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>22:13:12</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="n">
+        <v>31</v>
+      </c>
+      <c r="D13" s="33" t="n">
+        <v>91</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>870</v>
+      </c>
+      <c r="F13" s="33" t="n">
+        <v>42</v>
+      </c>
+      <c r="G13" s="33" t="n">
+        <v>226</v>
+      </c>
+      <c r="H13" s="33" t="n">
+        <v>474</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-02
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -867,7 +867,7 @@
     </row>
     <row r="13">
       <c r="A13" s="32" t="n">
-        <v>46266.92584414461</v>
+        <v>46266.92584414352</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -898,6 +898,44 @@
         </is>
       </c>
       <c r="J13" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="n">
+        <v>46267.92935670156</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>22:18:16</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" s="33" t="n">
+        <v>30</v>
+      </c>
+      <c r="E14" s="34" t="n">
+        <v>1029</v>
+      </c>
+      <c r="F14" s="33" t="n">
+        <v>85</v>
+      </c>
+      <c r="G14" s="33" t="n">
+        <v>44</v>
+      </c>
+      <c r="H14" s="33" t="n">
+        <v>18</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-03
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -905,7 +905,7 @@
     </row>
     <row r="14">
       <c r="A14" s="32" t="n">
-        <v>46267.92935670156</v>
+        <v>46267.92935670139</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -936,6 +936,44 @@
         </is>
       </c>
       <c r="J14" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="n">
+        <v>46268.92809245913</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>22:16:27</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="33" t="n">
+        <v>189</v>
+      </c>
+      <c r="E15" s="34" t="n">
+        <v>1188</v>
+      </c>
+      <c r="F15" s="33" t="n">
+        <v>244</v>
+      </c>
+      <c r="G15" s="33" t="n">
+        <v>203</v>
+      </c>
+      <c r="H15" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-04
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -943,7 +943,7 @@
     </row>
     <row r="15">
       <c r="A15" s="32" t="n">
-        <v>46268.92809245913</v>
+        <v>46268.9280924537</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -974,6 +974,44 @@
         </is>
       </c>
       <c r="J15" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="32" t="n">
+        <v>46269.9259836081</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>22:13:24</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="n">
+        <v>69</v>
+      </c>
+      <c r="D16" s="33" t="n">
+        <v>348</v>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>1347</v>
+      </c>
+      <c r="F16" s="33" t="n">
+        <v>81</v>
+      </c>
+      <c r="G16" s="33" t="n">
+        <v>362</v>
+      </c>
+      <c r="H16" s="33" t="n">
+        <v>37</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-05
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -981,7 +981,7 @@
     </row>
     <row r="16">
       <c r="A16" s="32" t="n">
-        <v>46269.9259836081</v>
+        <v>46269.92598361111</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1012,6 +1012,44 @@
         </is>
       </c>
       <c r="J16" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="32" t="n">
+        <v>46270.92538274504</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>22:12:33</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="n">
+        <v>228</v>
+      </c>
+      <c r="D17" s="33" t="n">
+        <v>507</v>
+      </c>
+      <c r="E17" s="33" t="n">
+        <v>62</v>
+      </c>
+      <c r="F17" s="33" t="n">
+        <v>72</v>
+      </c>
+      <c r="G17" s="34" t="n">
+        <v>521</v>
+      </c>
+      <c r="H17" s="33" t="n">
+        <v>29</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-06
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1019,7 +1019,7 @@
     </row>
     <row r="17">
       <c r="A17" s="32" t="n">
-        <v>46270.92538274504</v>
+        <v>46270.92538274306</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1050,6 +1050,44 @@
         </is>
       </c>
       <c r="J17" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="32" t="n">
+        <v>46271.92572152701</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>22:13:02</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="n">
+        <v>29</v>
+      </c>
+      <c r="D18" s="33" t="n">
+        <v>110</v>
+      </c>
+      <c r="E18" s="33" t="n">
+        <v>135</v>
+      </c>
+      <c r="F18" s="34" t="n">
+        <v>231</v>
+      </c>
+      <c r="G18" s="33" t="n">
+        <v>56</v>
+      </c>
+      <c r="H18" s="33" t="n">
+        <v>188</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-07
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1057,7 +1057,7 @@
     </row>
     <row r="18">
       <c r="A18" s="32" t="n">
-        <v>46271.92572152701</v>
+        <v>46271.92572152778</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1088,6 +1088,44 @@
         </is>
       </c>
       <c r="J18" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="n">
+        <v>46272.92604263419</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>22:13:30</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="n">
+        <v>188</v>
+      </c>
+      <c r="D19" s="33" t="n">
+        <v>269</v>
+      </c>
+      <c r="E19" s="33" t="n">
+        <v>294</v>
+      </c>
+      <c r="F19" s="34" t="n">
+        <v>390</v>
+      </c>
+      <c r="G19" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="33" t="n">
+        <v>29</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-08
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="19">
       <c r="A19" s="32" t="n">
-        <v>46272.92604263419</v>
+        <v>46272.92604263889</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1126,6 +1126,44 @@
         </is>
       </c>
       <c r="J19" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="32" t="n">
+        <v>46273.9273997625</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>22:15:27</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="n">
+        <v>46</v>
+      </c>
+      <c r="D20" s="33" t="n">
+        <v>428</v>
+      </c>
+      <c r="E20" s="34" t="n">
+        <v>453</v>
+      </c>
+      <c r="F20" s="33" t="n">
+        <v>29</v>
+      </c>
+      <c r="G20" s="33" t="n">
+        <v>85</v>
+      </c>
+      <c r="H20" s="33" t="n">
+        <v>188</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-09
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1133,7 +1133,7 @@
     </row>
     <row r="20">
       <c r="A20" s="32" t="n">
-        <v>46273.9273997625</v>
+        <v>46273.92739975695</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1164,6 +1164,44 @@
         </is>
       </c>
       <c r="J20" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="32" t="n">
+        <v>46274.92619760754</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>22:13:43</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="D21" s="34" t="n">
+        <v>587</v>
+      </c>
+      <c r="E21" s="33" t="n">
+        <v>97</v>
+      </c>
+      <c r="F21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="33" t="n">
+        <v>244</v>
+      </c>
+      <c r="H21" s="33" t="n">
+        <v>143</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-10
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="21">
       <c r="A21" s="32" t="n">
-        <v>46274.92619760754</v>
+        <v>46274.92619760417</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1202,6 +1202,44 @@
         </is>
       </c>
       <c r="J21" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="32" t="n">
+        <v>46275.92658699573</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>22:14:17</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="n">
+        <v>98</v>
+      </c>
+      <c r="D22" s="34" t="n">
+        <v>746</v>
+      </c>
+      <c r="E22" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="33" t="n">
+        <v>114</v>
+      </c>
+      <c r="G22" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="H22" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-11
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1209,7 +1209,7 @@
     </row>
     <row r="22">
       <c r="A22" s="32" t="n">
-        <v>46275.92658699573</v>
+        <v>46275.92658699074</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1240,6 +1240,44 @@
         </is>
       </c>
       <c r="J22" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="n">
+        <v>46276.92600875572</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>22:13:27</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="n">
+        <v>94</v>
+      </c>
+      <c r="D23" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="33" t="n">
+        <v>161</v>
+      </c>
+      <c r="F23" s="34" t="n">
+        <v>273</v>
+      </c>
+      <c r="G23" s="33" t="n">
+        <v>68</v>
+      </c>
+      <c r="H23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-12
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="23">
       <c r="A23" s="32" t="n">
-        <v>46276.92600875572</v>
+        <v>46276.92600875</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1278,6 +1278,44 @@
         </is>
       </c>
       <c r="J23" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="32" t="n">
+        <v>46277.92548483812</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>22:12:41</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="n">
+        <v>253</v>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="E24" s="33" t="n">
+        <v>77</v>
+      </c>
+      <c r="F24" s="34" t="n">
+        <v>432</v>
+      </c>
+      <c r="G24" s="33" t="n">
+        <v>73</v>
+      </c>
+      <c r="H24" s="33" t="n">
+        <v>133</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-13
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1285,7 +1285,7 @@
     </row>
     <row r="24">
       <c r="A24" s="32" t="n">
-        <v>46277.92548483812</v>
+        <v>46277.92548483796</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1316,6 +1316,44 @@
         </is>
       </c>
       <c r="J24" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32" t="n">
+        <v>46278.92586135297</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>22:13:14</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="n">
+        <v>55</v>
+      </c>
+      <c r="D25" s="33" t="n">
+        <v>51</v>
+      </c>
+      <c r="E25" s="33" t="n">
+        <v>236</v>
+      </c>
+      <c r="F25" s="34" t="n">
+        <v>591</v>
+      </c>
+      <c r="G25" s="33" t="n">
+        <v>232</v>
+      </c>
+      <c r="H25" s="33" t="n">
+        <v>292</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-14
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1323,7 +1323,7 @@
     </row>
     <row r="25">
       <c r="A25" s="32" t="n">
-        <v>46278.92586135297</v>
+        <v>46278.92586135417</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1354,6 +1354,44 @@
         </is>
       </c>
       <c r="J25" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="32" t="n">
+        <v>46279.92776884648</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>22:15:59</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="n">
+        <v>214</v>
+      </c>
+      <c r="D26" s="33" t="n">
+        <v>210</v>
+      </c>
+      <c r="E26" s="33" t="n">
+        <v>64</v>
+      </c>
+      <c r="F26" s="34" t="n">
+        <v>750</v>
+      </c>
+      <c r="G26" s="33" t="n">
+        <v>391</v>
+      </c>
+      <c r="H26" s="33" t="n">
+        <v>114</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-15
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1361,7 +1361,7 @@
     </row>
     <row r="26">
       <c r="A26" s="32" t="n">
-        <v>46279.92776884648</v>
+        <v>46279.92776884259</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1392,6 +1392,44 @@
         </is>
       </c>
       <c r="J26" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="n">
+        <v>46280.92606954329</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>22:13:32</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="n">
+        <v>373</v>
+      </c>
+      <c r="D27" s="33" t="n">
+        <v>369</v>
+      </c>
+      <c r="E27" s="33" t="n">
+        <v>128</v>
+      </c>
+      <c r="F27" s="34" t="n">
+        <v>909</v>
+      </c>
+      <c r="G27" s="33" t="n">
+        <v>134</v>
+      </c>
+      <c r="H27" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-16
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1399,7 +1399,7 @@
     </row>
     <row r="27">
       <c r="A27" s="32" t="n">
-        <v>46280.92606954329</v>
+        <v>46280.92606954861</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1430,6 +1430,44 @@
         </is>
       </c>
       <c r="J27" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="n">
+        <v>46281.92641638475</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>22:14:02</t>
+        </is>
+      </c>
+      <c r="C28" s="34" t="n">
+        <v>532</v>
+      </c>
+      <c r="D28" s="33" t="n">
+        <v>154</v>
+      </c>
+      <c r="E28" s="33" t="n">
+        <v>287</v>
+      </c>
+      <c r="F28" s="33" t="n">
+        <v>65</v>
+      </c>
+      <c r="G28" s="33" t="n">
+        <v>85</v>
+      </c>
+      <c r="H28" s="33" t="n">
+        <v>160</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-17
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1437,7 +1437,7 @@
     </row>
     <row r="28">
       <c r="A28" s="32" t="n">
-        <v>46281.92641638475</v>
+        <v>46281.92641638889</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1468,6 +1468,44 @@
         </is>
       </c>
       <c r="J28" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="32" t="n">
+        <v>46282.92687230668</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>22:14:41</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="n">
+        <v>62</v>
+      </c>
+      <c r="D29" s="33" t="n">
+        <v>313</v>
+      </c>
+      <c r="E29" s="33" t="n">
+        <v>57</v>
+      </c>
+      <c r="F29" s="33" t="n">
+        <v>224</v>
+      </c>
+      <c r="G29" s="33" t="n">
+        <v>244</v>
+      </c>
+      <c r="H29" s="34" t="n">
+        <v>319</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-18
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1475,7 +1475,7 @@
     </row>
     <row r="29">
       <c r="A29" s="32" t="n">
-        <v>46282.92687230668</v>
+        <v>46282.92687230324</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1506,6 +1506,44 @@
         </is>
       </c>
       <c r="J29" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="32" t="n">
+        <v>46283.92604304012</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>22:13:30</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="n">
+        <v>221</v>
+      </c>
+      <c r="D30" s="33" t="n">
+        <v>472</v>
+      </c>
+      <c r="E30" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" s="33" t="n">
+        <v>383</v>
+      </c>
+      <c r="G30" s="33" t="n">
+        <v>131</v>
+      </c>
+      <c r="H30" s="34" t="n">
+        <v>478</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-19
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1513,7 +1513,7 @@
     </row>
     <row r="30">
       <c r="A30" s="32" t="n">
-        <v>46283.92604304012</v>
+        <v>46283.92604304398</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1544,6 +1544,44 @@
         </is>
       </c>
       <c r="J30" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="32" t="n">
+        <v>46284.9252346662</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>22:12:20</t>
+        </is>
+      </c>
+      <c r="C31" s="33" t="n">
+        <v>131</v>
+      </c>
+      <c r="D31" s="33" t="n">
+        <v>76</v>
+      </c>
+      <c r="E31" s="33" t="n">
+        <v>127</v>
+      </c>
+      <c r="F31" s="33" t="n">
+        <v>125</v>
+      </c>
+      <c r="G31" s="33" t="n">
+        <v>14</v>
+      </c>
+      <c r="H31" s="34" t="n">
+        <v>637</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-20
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="31">
       <c r="A31" s="32" t="n">
-        <v>46284.9252346662</v>
+        <v>46284.92523466436</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1582,6 +1582,44 @@
         </is>
       </c>
       <c r="J31" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="n">
+        <v>46285.92551359671</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>22:12:44</t>
+        </is>
+      </c>
+      <c r="C32" s="34" t="n">
+        <v>290</v>
+      </c>
+      <c r="D32" s="33" t="n">
+        <v>235</v>
+      </c>
+      <c r="E32" s="33" t="n">
+        <v>24</v>
+      </c>
+      <c r="F32" s="33" t="n">
+        <v>32</v>
+      </c>
+      <c r="G32" s="33" t="n">
+        <v>119</v>
+      </c>
+      <c r="H32" s="33" t="n">
+        <v>71</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-21
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="32">
       <c r="A32" s="32" t="n">
-        <v>46285.92551359671</v>
+        <v>46285.92551359953</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1620,6 +1620,44 @@
         </is>
       </c>
       <c r="J32" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="n">
+        <v>46286.92553487718</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>22:12:46</t>
+        </is>
+      </c>
+      <c r="C33" s="34" t="n">
+        <v>449</v>
+      </c>
+      <c r="D33" s="33" t="n">
+        <v>394</v>
+      </c>
+      <c r="E33" s="33" t="n">
+        <v>183</v>
+      </c>
+      <c r="F33" s="33" t="n">
+        <v>191</v>
+      </c>
+      <c r="G33" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="H33" s="33" t="n">
+        <v>230</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-22
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1627,7 +1627,7 @@
     </row>
     <row r="33">
       <c r="A33" s="32" t="n">
-        <v>46286.92553487718</v>
+        <v>46286.92553487269</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1658,6 +1658,44 @@
         </is>
       </c>
       <c r="J33" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="n">
+        <v>46288.06726733701</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>01:36:51</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="n">
+        <v>31</v>
+      </c>
+      <c r="D34" s="34" t="n">
+        <v>553</v>
+      </c>
+      <c r="E34" s="33" t="n">
+        <v>342</v>
+      </c>
+      <c r="F34" s="33" t="n">
+        <v>57</v>
+      </c>
+      <c r="G34" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="H34" s="33" t="n">
+        <v>389</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-23
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1665,7 +1665,7 @@
     </row>
     <row r="34">
       <c r="A34" s="32" t="n">
-        <v>46288.06726733701</v>
+        <v>46288.06726733796</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1696,6 +1696,44 @@
         </is>
       </c>
       <c r="J34" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="n">
+        <v>46289.08002086973</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>01:55:13</t>
+        </is>
+      </c>
+      <c r="C35" s="33" t="n">
+        <v>115</v>
+      </c>
+      <c r="D35" s="33" t="n">
+        <v>57</v>
+      </c>
+      <c r="E35" s="34" t="n">
+        <v>500</v>
+      </c>
+      <c r="F35" s="33" t="n">
+        <v>140</v>
+      </c>
+      <c r="G35" s="33" t="n">
+        <v>171</v>
+      </c>
+      <c r="H35" s="33" t="n">
+        <v>154</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-24
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1703,7 +1703,7 @@
     </row>
     <row r="35">
       <c r="A35" s="32" t="n">
-        <v>46289.08002086973</v>
+        <v>46289.08002086805</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1734,6 +1734,44 @@
         </is>
       </c>
       <c r="J35" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="n">
+        <v>46290.0783057092</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>01:52:45</t>
+        </is>
+      </c>
+      <c r="C36" s="33" t="n">
+        <v>275</v>
+      </c>
+      <c r="D36" s="33" t="n">
+        <v>36</v>
+      </c>
+      <c r="E36" s="34" t="n">
+        <v>660</v>
+      </c>
+      <c r="F36" s="33" t="n">
+        <v>32</v>
+      </c>
+      <c r="G36" s="33" t="n">
+        <v>76</v>
+      </c>
+      <c r="H36" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-25
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1741,7 +1741,7 @@
     </row>
     <row r="36">
       <c r="A36" s="32" t="n">
-        <v>46290.0783057092</v>
+        <v>46290.07830570602</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1772,6 +1772,44 @@
         </is>
       </c>
       <c r="J36" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="n">
+        <v>46291.0904646585</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>02:10:16</t>
+        </is>
+      </c>
+      <c r="C37" s="33" t="n">
+        <v>434</v>
+      </c>
+      <c r="D37" s="33" t="n">
+        <v>195</v>
+      </c>
+      <c r="E37" s="34" t="n">
+        <v>819</v>
+      </c>
+      <c r="F37" s="33" t="n">
+        <v>153</v>
+      </c>
+      <c r="G37" s="33" t="n">
+        <v>33</v>
+      </c>
+      <c r="H37" s="33" t="n">
+        <v>166</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-26
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1779,7 +1779,7 @@
     </row>
     <row r="37">
       <c r="A37" s="32" t="n">
-        <v>46291.0904646585</v>
+        <v>46291.09046465278</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1810,6 +1810,44 @@
         </is>
       </c>
       <c r="J37" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="32" t="n">
+        <v>46292.05922454089</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>01:25:17</t>
+        </is>
+      </c>
+      <c r="C38" s="33" t="n">
+        <v>154</v>
+      </c>
+      <c r="D38" s="34" t="n">
+        <v>354</v>
+      </c>
+      <c r="E38" s="33" t="n">
+        <v>25</v>
+      </c>
+      <c r="F38" s="33" t="n">
+        <v>125</v>
+      </c>
+      <c r="G38" s="33" t="n">
+        <v>192</v>
+      </c>
+      <c r="H38" s="33" t="n">
+        <v>71</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-27
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1817,7 +1817,7 @@
     </row>
     <row r="38">
       <c r="A38" s="32" t="n">
-        <v>46292.05922454089</v>
+        <v>46292.05922453704</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1848,6 +1848,44 @@
         </is>
       </c>
       <c r="J38" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="32" t="n">
+        <v>46293.08055440612</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>01:55:59</t>
+        </is>
+      </c>
+      <c r="C39" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="D39" s="33" t="n">
+        <v>105</v>
+      </c>
+      <c r="E39" s="33" t="n">
+        <v>183</v>
+      </c>
+      <c r="F39" s="33" t="n">
+        <v>283</v>
+      </c>
+      <c r="G39" s="34" t="n">
+        <v>350</v>
+      </c>
+      <c r="H39" s="33" t="n">
+        <v>229</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-28
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1855,7 +1855,7 @@
     </row>
     <row r="39">
       <c r="A39" s="32" t="n">
-        <v>46293.08055440612</v>
+        <v>46293.08055440972</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1886,6 +1886,44 @@
         </is>
       </c>
       <c r="J39" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="32" t="n">
+        <v>46294.17203327677</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>04:07:43</t>
+        </is>
+      </c>
+      <c r="C40" s="33" t="n">
+        <v>152</v>
+      </c>
+      <c r="D40" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="33" t="n">
+        <v>158</v>
+      </c>
+      <c r="F40" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="G40" s="34" t="n">
+        <v>510</v>
+      </c>
+      <c r="H40" s="33" t="n">
+        <v>389</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-29
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1893,7 +1893,7 @@
     </row>
     <row r="40">
       <c r="A40" s="32" t="n">
-        <v>46294.17203327677</v>
+        <v>46294.17203327546</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1924,6 +1924,44 @@
         </is>
       </c>
       <c r="J40" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="32" t="n">
+        <v>46295.11933061467</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>02:51:50</t>
+        </is>
+      </c>
+      <c r="C41" s="33" t="n">
+        <v>311</v>
+      </c>
+      <c r="D41" s="33" t="n">
+        <v>162</v>
+      </c>
+      <c r="E41" s="34" t="n">
+        <v>317</v>
+      </c>
+      <c r="F41" s="33" t="n">
+        <v>14</v>
+      </c>
+      <c r="G41" s="33" t="n">
+        <v>117</v>
+      </c>
+      <c r="H41" s="33" t="n">
+        <v>96</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-09-30
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1931,7 +1931,7 @@
     </row>
     <row r="41">
       <c r="A41" s="32" t="n">
-        <v>46295.11933061467</v>
+        <v>46295.11933061342</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1962,6 +1962,44 @@
         </is>
       </c>
       <c r="J41" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="32" t="n">
+        <v>46296.12043094209</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>02:53:25</t>
+        </is>
+      </c>
+      <c r="C42" s="33" t="n">
+        <v>52</v>
+      </c>
+      <c r="D42" s="33" t="n">
+        <v>321</v>
+      </c>
+      <c r="E42" s="34" t="n">
+        <v>476</v>
+      </c>
+      <c r="F42" s="33" t="n">
+        <v>173</v>
+      </c>
+      <c r="G42" s="33" t="n">
+        <v>65</v>
+      </c>
+      <c r="H42" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-01
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="42">
       <c r="A42" s="32" t="n">
-        <v>46296.12043094209</v>
+        <v>46296.1204309375</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -2000,6 +2000,44 @@
         </is>
       </c>
       <c r="J42" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="32" t="n">
+        <v>46297.13343450619</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>03:12:08</t>
+        </is>
+      </c>
+      <c r="C43" s="34" t="n">
+        <v>211</v>
+      </c>
+      <c r="D43" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E43" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="F43" s="33" t="n">
+        <v>25</v>
+      </c>
+      <c r="G43" s="33" t="n">
+        <v>74</v>
+      </c>
+      <c r="H43" s="33" t="n">
+        <v>172</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-02
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2007,7 +2007,7 @@
     </row>
     <row r="43">
       <c r="A43" s="32" t="n">
-        <v>46297.13343450619</v>
+        <v>46297.13343450231</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -2038,6 +2038,44 @@
         </is>
       </c>
       <c r="J43" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="32" t="n">
+        <v>46298.11719351523</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>02:48:45</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="n">
+        <v>106</v>
+      </c>
+      <c r="D44" s="33" t="n">
+        <v>164</v>
+      </c>
+      <c r="E44" s="33" t="n">
+        <v>136</v>
+      </c>
+      <c r="F44" s="33" t="n">
+        <v>184</v>
+      </c>
+      <c r="G44" s="34" t="n">
+        <v>233</v>
+      </c>
+      <c r="H44" s="33" t="n">
+        <v>30</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-03
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2045,7 +2045,7 @@
     </row>
     <row r="44">
       <c r="A44" s="32" t="n">
-        <v>46298.11719351523</v>
+        <v>46298.11719351852</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2076,6 +2076,44 @@
         </is>
       </c>
       <c r="J44" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="32" t="n">
+        <v>46299.06578209021</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>01:34:43</t>
+        </is>
+      </c>
+      <c r="C45" s="33" t="n">
+        <v>35</v>
+      </c>
+      <c r="D45" s="33" t="n">
+        <v>323</v>
+      </c>
+      <c r="E45" s="33" t="n">
+        <v>74</v>
+      </c>
+      <c r="F45" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="34" t="n">
+        <v>392</v>
+      </c>
+      <c r="H45" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-04
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="45">
       <c r="A45" s="32" t="n">
-        <v>46299.06578209021</v>
+        <v>46299.06578209491</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2114,6 +2114,44 @@
         </is>
       </c>
       <c r="J45" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="32" t="n">
+        <v>46300.06509864423</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>01:33:44</t>
+        </is>
+      </c>
+      <c r="C46" s="33" t="n">
+        <v>55</v>
+      </c>
+      <c r="D46" s="33" t="n">
+        <v>482</v>
+      </c>
+      <c r="E46" s="33" t="n">
+        <v>156</v>
+      </c>
+      <c r="F46" s="33" t="n">
+        <v>160</v>
+      </c>
+      <c r="G46" s="34" t="n">
+        <v>551</v>
+      </c>
+      <c r="H46" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-05
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2121,7 +2121,7 @@
     </row>
     <row r="46">
       <c r="A46" s="32" t="n">
-        <v>46300.06509864423</v>
+        <v>46300.06509864583</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2152,6 +2152,44 @@
         </is>
       </c>
       <c r="J46" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="32" t="n">
+        <v>46301.20389764469</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>04:53:36</t>
+        </is>
+      </c>
+      <c r="C47" s="33" t="n">
+        <v>214</v>
+      </c>
+      <c r="D47" s="34" t="n">
+        <v>641</v>
+      </c>
+      <c r="E47" s="33" t="n">
+        <v>315</v>
+      </c>
+      <c r="F47" s="33" t="n">
+        <v>319</v>
+      </c>
+      <c r="G47" s="33" t="n">
+        <v>128</v>
+      </c>
+      <c r="H47" s="33" t="n">
+        <v>161</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-06
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2159,7 +2159,7 @@
     </row>
     <row r="47">
       <c r="A47" s="32" t="n">
-        <v>46301.20389764469</v>
+        <v>46301.20389765046</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2190,6 +2190,44 @@
         </is>
       </c>
       <c r="J47" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="32" t="n">
+        <v>46302.12814540699</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>03:04:31</t>
+        </is>
+      </c>
+      <c r="C48" s="33" t="n">
+        <v>106</v>
+      </c>
+      <c r="D48" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="E48" s="34" t="n">
+        <v>474</v>
+      </c>
+      <c r="F48" s="33" t="n">
+        <v>144</v>
+      </c>
+      <c r="G48" s="33" t="n">
+        <v>33</v>
+      </c>
+      <c r="H48" s="33" t="n">
+        <v>320</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-07
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2197,7 +2197,7 @@
     </row>
     <row r="48">
       <c r="A48" s="32" t="n">
-        <v>46302.12814540699</v>
+        <v>46302.12814540509</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2228,6 +2228,44 @@
         </is>
       </c>
       <c r="J48" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="32" t="n">
+        <v>46303.14551514522</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>03:29:32</t>
+        </is>
+      </c>
+      <c r="C49" s="33" t="n">
+        <v>28</v>
+      </c>
+      <c r="D49" s="33" t="n">
+        <v>172</v>
+      </c>
+      <c r="E49" s="34" t="n">
+        <v>633</v>
+      </c>
+      <c r="F49" s="33" t="n">
+        <v>24</v>
+      </c>
+      <c r="G49" s="33" t="n">
+        <v>192</v>
+      </c>
+      <c r="H49" s="33" t="n">
+        <v>479</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-08
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2235,7 +2235,7 @@
     </row>
     <row r="49">
       <c r="A49" s="32" t="n">
-        <v>46303.14551514522</v>
+        <v>46303.14551515046</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2266,6 +2266,44 @@
         </is>
       </c>
       <c r="J49" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="32" t="n">
+        <v>46304.14834123325</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>03:33:36</t>
+        </is>
+      </c>
+      <c r="C50" s="33" t="n">
+        <v>187</v>
+      </c>
+      <c r="D50" s="34" t="n">
+        <v>331</v>
+      </c>
+      <c r="E50" s="33" t="n">
+        <v>81</v>
+      </c>
+      <c r="F50" s="33" t="n">
+        <v>183</v>
+      </c>
+      <c r="G50" s="33" t="n">
+        <v>155</v>
+      </c>
+      <c r="H50" s="33" t="n">
+        <v>151</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-09
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2273,7 +2273,7 @@
     </row>
     <row r="50">
       <c r="A50" s="32" t="n">
-        <v>46304.14834123325</v>
+        <v>46304.14834123843</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2304,6 +2304,44 @@
         </is>
       </c>
       <c r="J50" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="32" t="n">
+        <v>46305.12626029671</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>03:01:48</t>
+        </is>
+      </c>
+      <c r="C51" s="33" t="n">
+        <v>30</v>
+      </c>
+      <c r="D51" s="33" t="n">
+        <v>89</v>
+      </c>
+      <c r="E51" s="33" t="n">
+        <v>85</v>
+      </c>
+      <c r="F51" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="G51" s="34" t="n">
+        <v>314</v>
+      </c>
+      <c r="H51" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-10
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2311,7 +2311,7 @@
     </row>
     <row r="51">
       <c r="A51" s="32" t="n">
-        <v>46305.12626029671</v>
+        <v>46305.12626030092</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -2342,6 +2342,44 @@
         </is>
       </c>
       <c r="J51" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="32" t="n">
+        <v>46306.09033525967</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>02:10:04</t>
+        </is>
+      </c>
+      <c r="C52" s="33" t="n">
+        <v>189</v>
+      </c>
+      <c r="D52" s="33" t="n">
+        <v>127</v>
+      </c>
+      <c r="E52" s="34" t="n">
+        <v>244</v>
+      </c>
+      <c r="F52" s="33" t="n">
+        <v>165</v>
+      </c>
+      <c r="G52" s="33" t="n">
+        <v>105</v>
+      </c>
+      <c r="H52" s="33" t="n">
+        <v>109</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-11
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2349,7 +2349,7 @@
     </row>
     <row r="52">
       <c r="A52" s="32" t="n">
-        <v>46306.09033525967</v>
+        <v>46306.09033525463</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2380,6 +2380,44 @@
         </is>
       </c>
       <c r="J52" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="32" t="n">
+        <v>46307.09997003007</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>02:23:57</t>
+        </is>
+      </c>
+      <c r="C53" s="34" t="n">
+        <v>348</v>
+      </c>
+      <c r="D53" s="33" t="n">
+        <v>68</v>
+      </c>
+      <c r="E53" s="33" t="n">
+        <v>70</v>
+      </c>
+      <c r="F53" s="33" t="n">
+        <v>125</v>
+      </c>
+      <c r="G53" s="33" t="n">
+        <v>63</v>
+      </c>
+      <c r="H53" s="33" t="n">
+        <v>47</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-12
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2387,7 +2387,7 @@
     </row>
     <row r="53">
       <c r="A53" s="32" t="n">
-        <v>46307.09997003007</v>
+        <v>46307.09997003472</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2418,6 +2418,44 @@
         </is>
       </c>
       <c r="J53" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="32" t="n">
+        <v>46308.22626826511</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>05:25:49</t>
+        </is>
+      </c>
+      <c r="C54" s="33" t="n">
+        <v>77</v>
+      </c>
+      <c r="D54" s="33" t="n">
+        <v>58</v>
+      </c>
+      <c r="E54" s="33" t="n">
+        <v>134</v>
+      </c>
+      <c r="F54" s="34" t="n">
+        <v>284</v>
+      </c>
+      <c r="G54" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="H54" s="33" t="n">
+        <v>206</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-13
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2425,7 +2425,7 @@
     </row>
     <row r="54">
       <c r="A54" s="32" t="n">
-        <v>46308.22626826511</v>
+        <v>46308.22626826389</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2456,6 +2456,44 @@
         </is>
       </c>
       <c r="J54" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="32" t="n">
+        <v>46309.14795384625</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>03:33:03</t>
+        </is>
+      </c>
+      <c r="C55" s="33" t="n">
+        <v>236</v>
+      </c>
+      <c r="D55" s="33" t="n">
+        <v>62</v>
+      </c>
+      <c r="E55" s="33" t="n">
+        <v>84</v>
+      </c>
+      <c r="F55" s="33" t="n">
+        <v>71</v>
+      </c>
+      <c r="G55" s="33" t="n">
+        <v>166</v>
+      </c>
+      <c r="H55" s="34" t="n">
+        <v>365</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-14
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -12,9 +12,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy hh:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -144,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -208,6 +209,7 @@
     <xf numFmtId="3" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -2463,30 +2465,28 @@
     </row>
     <row r="55">
       <c r="A55" s="32" t="n">
-        <v>46309.14795384625</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>03:33:03</t>
-        </is>
+        <v>46309</v>
+      </c>
+      <c r="B55" s="35" t="n">
+        <v>46309.35847963601</v>
       </c>
       <c r="C55" s="33" t="n">
-        <v>236</v>
+        <v>24</v>
       </c>
       <c r="D55" s="33" t="n">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="E55" s="33" t="n">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="F55" s="33" t="n">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="G55" s="33" t="n">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="H55" s="34" t="n">
-        <v>365</v>
+        <v>390</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-15
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -12,9 +12,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -482,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2465,10 +2466,10 @@
     </row>
     <row r="55">
       <c r="A55" s="32" t="n">
-        <v>46309.99240020317</v>
+        <v>46309.99240020834</v>
       </c>
       <c r="B55" s="36" t="n">
-        <v>46309.99240020317</v>
+        <v>46309.99240020834</v>
       </c>
       <c r="C55" s="33" t="n">
         <v>52</v>
@@ -2494,6 +2495,42 @@
         </is>
       </c>
       <c r="J55" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="32" t="n">
+        <v>46310.98278474271</v>
+      </c>
+      <c r="B56" s="36" t="n">
+        <v>46310.98278474271</v>
+      </c>
+      <c r="C56" s="33" t="n">
+        <v>211</v>
+      </c>
+      <c r="D56" s="33" t="n">
+        <v>197</v>
+      </c>
+      <c r="E56" s="33" t="n">
+        <v>40</v>
+      </c>
+      <c r="F56" s="33" t="n">
+        <v>42</v>
+      </c>
+      <c r="G56" s="34" t="n">
+        <v>484</v>
+      </c>
+      <c r="H56" s="33" t="n">
+        <v>229</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-16
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2502,10 +2502,10 @@
     </row>
     <row r="56">
       <c r="A56" s="32" t="n">
-        <v>46310.98278474271</v>
+        <v>46310.98278474537</v>
       </c>
       <c r="B56" s="36" t="n">
-        <v>46310.98278474271</v>
+        <v>46310.98278474537</v>
       </c>
       <c r="C56" s="33" t="n">
         <v>211</v>
@@ -2531,6 +2531,42 @@
         </is>
       </c>
       <c r="J56" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="32" t="n">
+        <v>46311.97208442223</v>
+      </c>
+      <c r="B57" s="36" t="n">
+        <v>46311.97208442223</v>
+      </c>
+      <c r="C57" s="33" t="n">
+        <v>64</v>
+      </c>
+      <c r="D57" s="33" t="n">
+        <v>52</v>
+      </c>
+      <c r="E57" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F57" s="33" t="n">
+        <v>125</v>
+      </c>
+      <c r="G57" s="34" t="n">
+        <v>643</v>
+      </c>
+      <c r="H57" s="33" t="n">
+        <v>388</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-17
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2538,10 +2538,10 @@
     </row>
     <row r="57">
       <c r="A57" s="32" t="n">
-        <v>46311.97208442223</v>
+        <v>46311.97208442129</v>
       </c>
       <c r="B57" s="36" t="n">
-        <v>46311.97208442223</v>
+        <v>46311.97208442129</v>
       </c>
       <c r="C57" s="33" t="n">
         <v>64</v>
@@ -2567,6 +2567,42 @@
         </is>
       </c>
       <c r="J57" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="32" t="n">
+        <v>46312.9265330889</v>
+      </c>
+      <c r="B58" s="36" t="n">
+        <v>46312.9265330889</v>
+      </c>
+      <c r="C58" s="33" t="n">
+        <v>29</v>
+      </c>
+      <c r="D58" s="33" t="n">
+        <v>21</v>
+      </c>
+      <c r="E58" s="33" t="n">
+        <v>165</v>
+      </c>
+      <c r="F58" s="33" t="n">
+        <v>62</v>
+      </c>
+      <c r="G58" s="33" t="n">
+        <v>20</v>
+      </c>
+      <c r="H58" s="34" t="n">
+        <v>547</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-18
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2574,10 +2574,10 @@
     </row>
     <row r="58">
       <c r="A58" s="32" t="n">
-        <v>46312.9265330889</v>
+        <v>46312.92653309028</v>
       </c>
       <c r="B58" s="36" t="n">
-        <v>46312.9265330889</v>
+        <v>46312.92653309028</v>
       </c>
       <c r="C58" s="33" t="n">
         <v>29</v>
@@ -2603,6 +2603,42 @@
         </is>
       </c>
       <c r="J58" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="32" t="n">
+        <v>46313.94150319308</v>
+      </c>
+      <c r="B59" s="36" t="n">
+        <v>46313.94150319308</v>
+      </c>
+      <c r="C59" s="33" t="n">
+        <v>188</v>
+      </c>
+      <c r="D59" s="33" t="n">
+        <v>180</v>
+      </c>
+      <c r="E59" s="33" t="n">
+        <v>118</v>
+      </c>
+      <c r="F59" s="33" t="n">
+        <v>154</v>
+      </c>
+      <c r="G59" s="33" t="n">
+        <v>179</v>
+      </c>
+      <c r="H59" s="34" t="n">
+        <v>706</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-20
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2610,10 +2610,10 @@
     </row>
     <row r="59">
       <c r="A59" s="32" t="n">
-        <v>46313.94150319308</v>
+        <v>46313.94150319444</v>
       </c>
       <c r="B59" s="36" t="n">
-        <v>46313.94150319308</v>
+        <v>46313.94150319444</v>
       </c>
       <c r="C59" s="33" t="n">
         <v>188</v>
@@ -2639,6 +2639,42 @@
         </is>
       </c>
       <c r="J59" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="32" t="n">
+        <v>46315.98226920456</v>
+      </c>
+      <c r="B60" s="36" t="n">
+        <v>46315.98226920456</v>
+      </c>
+      <c r="C60" s="34" t="n">
+        <v>506</v>
+      </c>
+      <c r="D60" s="33" t="n">
+        <v>40</v>
+      </c>
+      <c r="E60" s="33" t="n">
+        <v>127</v>
+      </c>
+      <c r="F60" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="G60" s="33" t="n">
+        <v>114</v>
+      </c>
+      <c r="H60" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-21
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2646,10 +2646,10 @@
     </row>
     <row r="60">
       <c r="A60" s="32" t="n">
-        <v>46315.98226920456</v>
+        <v>46315.98226920139</v>
       </c>
       <c r="B60" s="36" t="n">
-        <v>46315.98226920456</v>
+        <v>46315.98226920139</v>
       </c>
       <c r="C60" s="34" t="n">
         <v>506</v>
@@ -2675,6 +2675,42 @@
         </is>
       </c>
       <c r="J60" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="32" t="n">
+        <v>46316.99457137511</v>
+      </c>
+      <c r="B61" s="36" t="n">
+        <v>46316.99457137511</v>
+      </c>
+      <c r="C61" s="33" t="n">
+        <v>130</v>
+      </c>
+      <c r="D61" s="33" t="n">
+        <v>86</v>
+      </c>
+      <c r="E61" s="34" t="n">
+        <v>286</v>
+      </c>
+      <c r="F61" s="33" t="n">
+        <v>106</v>
+      </c>
+      <c r="G61" s="33" t="n">
+        <v>273</v>
+      </c>
+      <c r="H61" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-22
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2682,10 +2682,10 @@
     </row>
     <row r="61">
       <c r="A61" s="32" t="n">
-        <v>46316.99457137511</v>
+        <v>46316.99457137731</v>
       </c>
       <c r="B61" s="36" t="n">
-        <v>46316.99457137511</v>
+        <v>46316.99457137731</v>
       </c>
       <c r="C61" s="33" t="n">
         <v>130</v>
@@ -2711,6 +2711,42 @@
         </is>
       </c>
       <c r="J61" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="32" t="n">
+        <v>46317.9947263709</v>
+      </c>
+      <c r="B62" s="36" t="n">
+        <v>46317.9947263709</v>
+      </c>
+      <c r="C62" s="33" t="n">
+        <v>145</v>
+      </c>
+      <c r="D62" s="33" t="n">
+        <v>245</v>
+      </c>
+      <c r="E62" s="34" t="n">
+        <v>445</v>
+      </c>
+      <c r="F62" s="33" t="n">
+        <v>265</v>
+      </c>
+      <c r="G62" s="33" t="n">
+        <v>80</v>
+      </c>
+      <c r="H62" s="33" t="n">
+        <v>162</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-23
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2718,10 +2718,10 @@
     </row>
     <row r="62">
       <c r="A62" s="32" t="n">
-        <v>46317.9947263709</v>
+        <v>46317.99472636574</v>
       </c>
       <c r="B62" s="36" t="n">
-        <v>46317.9947263709</v>
+        <v>46317.99472636574</v>
       </c>
       <c r="C62" s="33" t="n">
         <v>145</v>
@@ -2747,6 +2747,42 @@
         </is>
       </c>
       <c r="J62" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="32" t="n">
+        <v>46318.98877453398</v>
+      </c>
+      <c r="B63" s="36" t="n">
+        <v>46318.98877453398</v>
+      </c>
+      <c r="C63" s="33" t="n">
+        <v>304</v>
+      </c>
+      <c r="D63" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E63" s="34" t="n">
+        <v>604</v>
+      </c>
+      <c r="F63" s="33" t="n">
+        <v>123</v>
+      </c>
+      <c r="G63" s="33" t="n">
+        <v>239</v>
+      </c>
+      <c r="H63" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-24
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2754,10 +2754,10 @@
     </row>
     <row r="63">
       <c r="A63" s="32" t="n">
-        <v>46318.98877453398</v>
+        <v>46318.98877453704</v>
       </c>
       <c r="B63" s="36" t="n">
-        <v>46318.98877453398</v>
+        <v>46318.98877453704</v>
       </c>
       <c r="C63" s="33" t="n">
         <v>304</v>
@@ -2783,6 +2783,42 @@
         </is>
       </c>
       <c r="J63" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="32" t="n">
+        <v>46319.94235838785</v>
+      </c>
+      <c r="B64" s="36" t="n">
+        <v>46319.94235838785</v>
+      </c>
+      <c r="C64" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="33" t="n">
+        <v>70</v>
+      </c>
+      <c r="E64" s="34" t="n">
+        <v>763</v>
+      </c>
+      <c r="F64" s="33" t="n">
+        <v>77</v>
+      </c>
+      <c r="G64" s="33" t="n">
+        <v>63</v>
+      </c>
+      <c r="H64" s="33" t="n">
+        <v>159</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>

<commit_message>
Cap nhat Tam hoa 2026-10-25
</commit_message>
<xml_diff>
--- a/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
+++ b/github_bingo18/Bingo18_Lich_su_Tam_hoa.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2790,10 +2790,10 @@
     </row>
     <row r="64">
       <c r="A64" s="32" t="n">
-        <v>46319.94235838785</v>
+        <v>46319.94235839121</v>
       </c>
       <c r="B64" s="36" t="n">
-        <v>46319.94235838785</v>
+        <v>46319.94235839121</v>
       </c>
       <c r="C64" s="33" t="n">
         <v>0</v>
@@ -2819,6 +2819,42 @@
         </is>
       </c>
       <c r="J64" t="inlineStr">
+        <is>
+          <t>Thành công - Kết nối bảo mật bình thường</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="32" t="n">
+        <v>46320.94974142367</v>
+      </c>
+      <c r="B65" s="36" t="n">
+        <v>46320.94974142367</v>
+      </c>
+      <c r="C65" s="33" t="n">
+        <v>159</v>
+      </c>
+      <c r="D65" s="33" t="n">
+        <v>83</v>
+      </c>
+      <c r="E65" s="34" t="n">
+        <v>922</v>
+      </c>
+      <c r="F65" s="33" t="n">
+        <v>236</v>
+      </c>
+      <c r="G65" s="33" t="n">
+        <v>35</v>
+      </c>
+      <c r="H65" s="33" t="n">
+        <v>18</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>https://www.bingo18.top/data/data.json</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
         <is>
           <t>Thành công - Kết nối bảo mật bình thường</t>
         </is>

</xml_diff>